<commit_message>
updates to raw data files
</commit_message>
<xml_diff>
--- a/data/raw/GLNPO 2024 Spring/Erie/D100/ER 63 D100 Spring 202424GE00I33 Zoops.xlsx
+++ b/data/raw/GLNPO 2024 Spring/Erie/D100/ER 63 D100 Spring 202424GE00I33 Zoops.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27928"/>
   <workbookPr hidePivotFieldList="1" defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\cmars\OneDrive\Desktop\CCM Work Files\GLNPO Zooplankton Database\data\raw\GLNPO 2024 Spring\Erie\D100\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\GL Lab User\Desktop\GLNPO Sample Files\2024\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BE6E3ED7-F332-44B3-A0F9-B2B11091E195}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{05CF88FB-4B0A-4E99-8E6B-B73FD8E6313D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="11424" yWindow="0" windowWidth="11712" windowHeight="12336" xr2:uid="{5EC08AF0-3BF1-4A72-9C0A-B465BE7095BF}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17640" xr2:uid="{5EC08AF0-3BF1-4A72-9C0A-B465BE7095BF}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -18,9 +18,9 @@
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sheet1!$A$1:$R$205</definedName>
   </definedNames>
-  <calcPr calcId="191029"/>
+  <calcPr calcId="191029" concurrentCalc="0"/>
   <pivotCaches>
-    <pivotCache cacheId="10" r:id="rId2"/>
+    <pivotCache cacheId="620" r:id="rId2"/>
   </pivotCaches>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
@@ -466,7 +466,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="1" applyNumberFormat="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="15">
+  <cellXfs count="16">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -475,17 +475,18 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="14" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="7" fillId="3" borderId="1" xfId="1" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="1" xfId="1" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -4498,7 +4499,7 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable1.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{94D0AD5D-9AD0-4F8A-B5BC-0E7B4216228B}" name="PivotTable1" cacheId="10" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{94D0AD5D-9AD0-4F8A-B5BC-0E7B4216228B}" name="PivotTable1" cacheId="620" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
   <location ref="U2:Z19" firstHeaderRow="1" firstDataRow="2" firstDataCol="1"/>
   <pivotFields count="17">
     <pivotField showAll="0"/>
@@ -4952,22 +4953,22 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6FCF592D-064A-4BB8-8378-1CCFC4766115}">
   <dimension ref="A1:Z205"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="4" max="4" width="9.33203125" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="9.33203125" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="9.44140625" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="31.88671875" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="9.33203125" bestFit="1" customWidth="1"/>
-    <col min="21" max="21" width="31.88671875" bestFit="1" customWidth="1"/>
-    <col min="22" max="22" width="16.88671875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="9.28515625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="9.28515625" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="9.42578125" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="31.85546875" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="9.28515625" bestFit="1" customWidth="1"/>
+    <col min="21" max="21" width="31.85546875" bestFit="1" customWidth="1"/>
+    <col min="22" max="22" width="16.85546875" bestFit="1" customWidth="1"/>
     <col min="23" max="23" width="4" bestFit="1" customWidth="1"/>
     <col min="24" max="24" width="3" bestFit="1" customWidth="1"/>
-    <col min="25" max="25" width="7.33203125" bestFit="1" customWidth="1"/>
-    <col min="26" max="26" width="11.33203125" bestFit="1" customWidth="1"/>
+    <col min="25" max="25" width="7.28515625" bestFit="1" customWidth="1"/>
+    <col min="26" max="26" width="11.28515625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:26" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -5023,7 +5024,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="2" spans="1:26" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>18</v>
       </c>
@@ -5082,7 +5083,7 @@
         <v>73</v>
       </c>
     </row>
-    <row r="3" spans="1:26" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>18</v>
       </c>
@@ -5153,7 +5154,7 @@
         <v>71</v>
       </c>
     </row>
-    <row r="4" spans="1:26" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>18</v>
       </c>
@@ -5208,17 +5209,19 @@
       <c r="U4" s="5" t="s">
         <v>25</v>
       </c>
-      <c r="V4">
+      <c r="V4" s="6">
         <v>58</v>
       </c>
-      <c r="W4">
+      <c r="W4" s="6">
         <v>50</v>
       </c>
-      <c r="Z4">
+      <c r="X4" s="6"/>
+      <c r="Y4" s="6"/>
+      <c r="Z4" s="6">
         <v>108</v>
       </c>
     </row>
-    <row r="5" spans="1:26" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>18</v>
       </c>
@@ -5273,17 +5276,19 @@
       <c r="U5" s="5" t="s">
         <v>42</v>
       </c>
-      <c r="V5">
+      <c r="V5" s="6">
         <v>40</v>
       </c>
-      <c r="W5">
+      <c r="W5" s="6">
         <v>57</v>
       </c>
-      <c r="Z5">
+      <c r="X5" s="6"/>
+      <c r="Y5" s="6"/>
+      <c r="Z5" s="6">
         <v>97</v>
       </c>
     </row>
-    <row r="6" spans="1:26" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>18</v>
       </c>
@@ -5338,20 +5343,21 @@
       <c r="U6" s="5" t="s">
         <v>53</v>
       </c>
-      <c r="V6">
+      <c r="V6" s="6">
         <v>3</v>
       </c>
-      <c r="W6">
+      <c r="W6" s="6">
         <v>5</v>
       </c>
-      <c r="X6">
+      <c r="X6" s="6">
         <v>4</v>
       </c>
-      <c r="Z6">
+      <c r="Y6" s="6"/>
+      <c r="Z6" s="6">
         <v>12</v>
       </c>
     </row>
-    <row r="7" spans="1:26" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>18</v>
       </c>
@@ -5406,20 +5412,21 @@
       <c r="U7" s="5" t="s">
         <v>59</v>
       </c>
-      <c r="V7">
-        <v>1</v>
-      </c>
-      <c r="W7">
+      <c r="V7" s="6">
+        <v>1</v>
+      </c>
+      <c r="W7" s="6">
         <v>0</v>
       </c>
-      <c r="X7">
-        <v>1</v>
-      </c>
-      <c r="Z7">
+      <c r="X7" s="6">
+        <v>1</v>
+      </c>
+      <c r="Y7" s="6"/>
+      <c r="Z7" s="6">
         <v>2</v>
       </c>
     </row>
-    <row r="8" spans="1:26" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>18</v>
       </c>
@@ -5474,20 +5481,21 @@
       <c r="U8" s="5" t="s">
         <v>30</v>
       </c>
-      <c r="V8">
+      <c r="V8" s="6">
         <v>9</v>
       </c>
-      <c r="W8">
+      <c r="W8" s="6">
         <v>4</v>
       </c>
-      <c r="X8">
+      <c r="X8" s="6">
         <v>13</v>
       </c>
-      <c r="Z8">
+      <c r="Y8" s="6"/>
+      <c r="Z8" s="6">
         <v>26</v>
       </c>
     </row>
-    <row r="9" spans="1:26" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>18</v>
       </c>
@@ -5542,17 +5550,19 @@
       <c r="U9" s="5" t="s">
         <v>38</v>
       </c>
-      <c r="V9">
+      <c r="V9" s="6">
         <v>74</v>
       </c>
-      <c r="W9">
+      <c r="W9" s="6">
         <v>72</v>
       </c>
-      <c r="Z9">
+      <c r="X9" s="6"/>
+      <c r="Y9" s="6"/>
+      <c r="Z9" s="6">
         <v>146</v>
       </c>
     </row>
-    <row r="10" spans="1:26" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>18</v>
       </c>
@@ -5607,20 +5617,21 @@
       <c r="U10" s="5" t="s">
         <v>49</v>
       </c>
-      <c r="V10">
+      <c r="V10" s="6">
         <v>2</v>
       </c>
-      <c r="W10">
-        <v>1</v>
-      </c>
-      <c r="X10">
+      <c r="W10" s="6">
+        <v>1</v>
+      </c>
+      <c r="X10" s="6">
         <v>0</v>
       </c>
-      <c r="Z10">
+      <c r="Y10" s="6"/>
+      <c r="Z10" s="6">
         <v>3</v>
       </c>
     </row>
-    <row r="11" spans="1:26" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>18</v>
       </c>
@@ -5675,20 +5686,21 @@
       <c r="U11" s="5" t="s">
         <v>67</v>
       </c>
-      <c r="V11">
+      <c r="V11" s="6">
         <v>0</v>
       </c>
-      <c r="W11">
+      <c r="W11" s="6">
         <v>0</v>
       </c>
-      <c r="X11">
+      <c r="X11" s="6">
         <v>3</v>
       </c>
-      <c r="Z11">
+      <c r="Y11" s="6"/>
+      <c r="Z11" s="6">
         <v>3</v>
       </c>
     </row>
-    <row r="12" spans="1:26" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>18</v>
       </c>
@@ -5743,20 +5755,21 @@
       <c r="U12" s="5" t="s">
         <v>51</v>
       </c>
-      <c r="V12">
+      <c r="V12" s="6">
         <v>2</v>
       </c>
-      <c r="W12">
-        <v>1</v>
-      </c>
-      <c r="X12">
-        <v>1</v>
-      </c>
-      <c r="Z12">
+      <c r="W12" s="6">
+        <v>1</v>
+      </c>
+      <c r="X12" s="6">
+        <v>1</v>
+      </c>
+      <c r="Y12" s="6"/>
+      <c r="Z12" s="6">
         <v>4</v>
       </c>
     </row>
-    <row r="13" spans="1:26" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>18</v>
       </c>
@@ -5811,20 +5824,21 @@
       <c r="U13" s="5" t="s">
         <v>46</v>
       </c>
-      <c r="V13">
+      <c r="V13" s="6">
         <v>5</v>
       </c>
-      <c r="W13">
+      <c r="W13" s="6">
         <v>0</v>
       </c>
-      <c r="X13">
+      <c r="X13" s="6">
         <v>0</v>
       </c>
-      <c r="Z13">
+      <c r="Y13" s="6"/>
+      <c r="Z13" s="6">
         <v>5</v>
       </c>
     </row>
-    <row r="14" spans="1:26" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>18</v>
       </c>
@@ -5879,20 +5893,21 @@
       <c r="U14" s="5" t="s">
         <v>62</v>
       </c>
-      <c r="V14">
+      <c r="V14" s="6">
         <v>0</v>
       </c>
-      <c r="W14">
+      <c r="W14" s="6">
         <v>2</v>
       </c>
-      <c r="X14">
+      <c r="X14" s="6">
         <v>0</v>
       </c>
-      <c r="Z14">
+      <c r="Y14" s="6"/>
+      <c r="Z14" s="6">
         <v>2</v>
       </c>
     </row>
-    <row r="15" spans="1:26" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
         <v>18</v>
       </c>
@@ -5947,20 +5962,21 @@
       <c r="U15" s="5" t="s">
         <v>65</v>
       </c>
-      <c r="V15">
+      <c r="V15" s="6">
         <v>0</v>
       </c>
-      <c r="W15">
+      <c r="W15" s="6">
         <v>0</v>
       </c>
-      <c r="X15">
-        <v>1</v>
-      </c>
-      <c r="Z15">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="16" spans="1:26" x14ac:dyDescent="0.3">
+      <c r="X15" s="6">
+        <v>1</v>
+      </c>
+      <c r="Y15" s="6"/>
+      <c r="Z15" s="6">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="16" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
         <v>18</v>
       </c>
@@ -6015,17 +6031,19 @@
       <c r="U16" s="5" t="s">
         <v>33</v>
       </c>
-      <c r="V16">
+      <c r="V16" s="6">
         <v>40</v>
       </c>
-      <c r="W16">
+      <c r="W16" s="6">
         <v>54</v>
       </c>
-      <c r="Z16">
+      <c r="X16" s="6"/>
+      <c r="Y16" s="6"/>
+      <c r="Z16" s="6">
         <v>94</v>
       </c>
     </row>
-    <row r="17" spans="1:26" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
         <v>18</v>
       </c>
@@ -6080,20 +6098,21 @@
       <c r="U17" s="5" t="s">
         <v>56</v>
       </c>
-      <c r="V17">
+      <c r="V17" s="6">
         <v>2</v>
       </c>
-      <c r="W17">
+      <c r="W17" s="6">
         <v>0</v>
       </c>
-      <c r="X17">
+      <c r="X17" s="6">
         <v>0</v>
       </c>
-      <c r="Z17">
+      <c r="Y17" s="6"/>
+      <c r="Z17" s="6">
         <v>2</v>
       </c>
     </row>
-    <row r="18" spans="1:26" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
         <v>18</v>
       </c>
@@ -6148,8 +6167,13 @@
       <c r="U18" s="5" t="s">
         <v>70</v>
       </c>
-    </row>
-    <row r="19" spans="1:26" x14ac:dyDescent="0.3">
+      <c r="V18" s="6"/>
+      <c r="W18" s="6"/>
+      <c r="X18" s="6"/>
+      <c r="Y18" s="6"/>
+      <c r="Z18" s="6"/>
+    </row>
+    <row r="19" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
         <v>18</v>
       </c>
@@ -6204,20 +6228,21 @@
       <c r="U19" s="5" t="s">
         <v>71</v>
       </c>
-      <c r="V19">
+      <c r="V19" s="6">
         <v>236</v>
       </c>
-      <c r="W19">
+      <c r="W19" s="6">
         <v>246</v>
       </c>
-      <c r="X19">
-        <v>23</v>
-      </c>
-      <c r="Z19">
+      <c r="X19" s="6">
+        <v>23</v>
+      </c>
+      <c r="Y19" s="6"/>
+      <c r="Z19" s="6">
         <v>505</v>
       </c>
     </row>
-    <row r="20" spans="1:26" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
         <v>18</v>
       </c>
@@ -6270,7 +6295,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="21" spans="1:26" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:26" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
         <v>18</v>
       </c>
@@ -6322,17 +6347,17 @@
       <c r="Q21">
         <v>1</v>
       </c>
-      <c r="U21" s="11" t="s">
+      <c r="U21" s="9" t="s">
         <v>74</v>
       </c>
-      <c r="V21" s="8" t="s">
+      <c r="V21" s="10" t="s">
         <v>75</v>
       </c>
-      <c r="W21" s="9">
+      <c r="W21" s="11">
         <v>0.999</v>
       </c>
     </row>
-    <row r="22" spans="1:26" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:26" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
         <v>18</v>
       </c>
@@ -6385,14 +6410,14 @@
         <v>1</v>
       </c>
       <c r="U22" s="12"/>
-      <c r="V22" s="8" t="s">
+      <c r="V22" s="10" t="s">
         <v>75</v>
       </c>
-      <c r="W22" s="9">
+      <c r="W22" s="11">
         <v>1.002</v>
       </c>
     </row>
-    <row r="23" spans="1:26" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:26" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
         <v>18</v>
       </c>
@@ -6444,17 +6469,17 @@
       <c r="Q23">
         <v>1</v>
       </c>
-      <c r="U23" s="11" t="s">
+      <c r="U23" s="9" t="s">
         <v>76</v>
       </c>
-      <c r="V23" s="8" t="s">
+      <c r="V23" s="10" t="s">
         <v>75</v>
       </c>
-      <c r="W23" s="9">
+      <c r="W23" s="11">
         <v>0.999</v>
       </c>
     </row>
-    <row r="24" spans="1:26" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:26" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
         <v>18</v>
       </c>
@@ -6507,14 +6532,14 @@
         <v>1</v>
       </c>
       <c r="U24" s="12"/>
-      <c r="V24" s="8" t="s">
+      <c r="V24" s="10" t="s">
         <v>75</v>
       </c>
-      <c r="W24" s="9">
+      <c r="W24" s="11">
         <v>0.996</v>
       </c>
     </row>
-    <row r="25" spans="1:26" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:26" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
         <v>18</v>
       </c>
@@ -6566,15 +6591,15 @@
       <c r="Q25">
         <v>1</v>
       </c>
-      <c r="U25" s="10" t="s">
+      <c r="U25" s="13" t="s">
         <v>77</v>
       </c>
-      <c r="V25" s="13" t="s">
+      <c r="V25" s="14" t="s">
         <v>78</v>
       </c>
-      <c r="W25" s="14"/>
-    </row>
-    <row r="26" spans="1:26" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="W25" s="15"/>
+    </row>
+    <row r="26" spans="1:26" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
         <v>18</v>
       </c>
@@ -6626,15 +6651,15 @@
       <c r="Q26">
         <v>1</v>
       </c>
-      <c r="U26" s="10" t="s">
+      <c r="U26" s="13" t="s">
         <v>79</v>
       </c>
-      <c r="V26" s="13" t="s">
+      <c r="V26" s="14" t="s">
         <v>80</v>
       </c>
-      <c r="W26" s="14"/>
-    </row>
-    <row r="27" spans="1:26" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="W26" s="15"/>
+    </row>
+    <row r="27" spans="1:26" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
         <v>18</v>
       </c>
@@ -6686,15 +6711,15 @@
       <c r="Q27">
         <v>1</v>
       </c>
-      <c r="U27" s="8" t="s">
+      <c r="U27" s="10" t="s">
         <v>81</v>
       </c>
-      <c r="V27" s="13" t="s">
+      <c r="V27" s="14" t="s">
         <v>82</v>
       </c>
-      <c r="W27" s="14"/>
-    </row>
-    <row r="28" spans="1:26" x14ac:dyDescent="0.3">
+      <c r="W27" s="15"/>
+    </row>
+    <row r="28" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
         <v>18</v>
       </c>
@@ -6747,7 +6772,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="29" spans="1:26" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
         <v>18</v>
       </c>
@@ -6800,7 +6825,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="30" spans="1:26" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
         <v>18</v>
       </c>
@@ -6853,7 +6878,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="31" spans="1:26" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
         <v>18</v>
       </c>
@@ -6906,7 +6931,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="32" spans="1:26" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
         <v>18</v>
       </c>
@@ -6959,7 +6984,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="33" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
         <v>18</v>
       </c>
@@ -7012,7 +7037,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="34" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
         <v>18</v>
       </c>
@@ -7065,7 +7090,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="35" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="35" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
         <v>18</v>
       </c>
@@ -7118,7 +7143,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="36" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="36" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
         <v>18</v>
       </c>
@@ -7171,7 +7196,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="37" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="37" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
         <v>18</v>
       </c>
@@ -7224,7 +7249,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="38" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="38" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
         <v>18</v>
       </c>
@@ -7277,7 +7302,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="39" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="39" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
         <v>18</v>
       </c>
@@ -7330,7 +7355,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="40" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="40" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
         <v>18</v>
       </c>
@@ -7383,7 +7408,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="41" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="41" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
         <v>18</v>
       </c>
@@ -7436,7 +7461,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="42" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="42" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
         <v>18</v>
       </c>
@@ -7489,7 +7514,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="43" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="43" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A43" t="s">
         <v>18</v>
       </c>
@@ -7542,7 +7567,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="44" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="44" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A44" t="s">
         <v>18</v>
       </c>
@@ -7595,7 +7620,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="45" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="45" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A45" t="s">
         <v>18</v>
       </c>
@@ -7648,7 +7673,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="46" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="46" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A46" t="s">
         <v>18</v>
       </c>
@@ -7701,7 +7726,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="47" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="47" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A47" t="s">
         <v>18</v>
       </c>
@@ -7754,7 +7779,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="48" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="48" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A48" t="s">
         <v>18</v>
       </c>
@@ -7807,7 +7832,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="49" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="49" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A49" t="s">
         <v>18</v>
       </c>
@@ -7860,7 +7885,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="50" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="50" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A50" t="s">
         <v>18</v>
       </c>
@@ -7913,7 +7938,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="51" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="51" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A51" t="s">
         <v>18</v>
       </c>
@@ -7966,7 +7991,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="52" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="52" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A52" t="s">
         <v>18</v>
       </c>
@@ -8019,7 +8044,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="53" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="53" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A53" t="s">
         <v>18</v>
       </c>
@@ -8072,7 +8097,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="54" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="54" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A54" t="s">
         <v>18</v>
       </c>
@@ -8128,7 +8153,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="55" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="55" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A55" t="s">
         <v>18</v>
       </c>
@@ -8181,7 +8206,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="56" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="56" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A56" t="s">
         <v>18</v>
       </c>
@@ -8234,7 +8259,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="57" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="57" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A57" t="s">
         <v>18</v>
       </c>
@@ -8287,7 +8312,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="58" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="58" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A58" t="s">
         <v>18</v>
       </c>
@@ -8340,7 +8365,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="59" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="59" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A59" t="s">
         <v>18</v>
       </c>
@@ -8393,7 +8418,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="60" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="60" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A60" t="s">
         <v>18</v>
       </c>
@@ -8446,7 +8471,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="61" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="61" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A61" t="s">
         <v>18</v>
       </c>
@@ -8499,7 +8524,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="62" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="62" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A62" t="s">
         <v>18</v>
       </c>
@@ -8552,7 +8577,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="63" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="63" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A63" t="s">
         <v>18</v>
       </c>
@@ -8605,7 +8630,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="64" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="64" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A64" t="s">
         <v>18</v>
       </c>
@@ -8658,7 +8683,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="65" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="65" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A65" t="s">
         <v>18</v>
       </c>
@@ -8711,7 +8736,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="66" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="66" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A66" t="s">
         <v>18</v>
       </c>
@@ -8764,7 +8789,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="67" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="67" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A67" t="s">
         <v>18</v>
       </c>
@@ -8817,7 +8842,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="68" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="68" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A68" t="s">
         <v>18</v>
       </c>
@@ -8870,7 +8895,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="69" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="69" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A69" t="s">
         <v>18</v>
       </c>
@@ -8923,7 +8948,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="70" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="70" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A70" t="s">
         <v>18</v>
       </c>
@@ -8976,7 +9001,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="71" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="71" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A71" t="s">
         <v>18</v>
       </c>
@@ -9029,7 +9054,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="72" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="72" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A72" t="s">
         <v>18</v>
       </c>
@@ -9082,7 +9107,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="73" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="73" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A73" t="s">
         <v>18</v>
       </c>
@@ -9135,7 +9160,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="74" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="74" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A74" t="s">
         <v>18</v>
       </c>
@@ -9188,7 +9213,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="75" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="75" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A75" t="s">
         <v>18</v>
       </c>
@@ -9241,7 +9266,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="76" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="76" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A76" t="s">
         <v>18</v>
       </c>
@@ -9294,7 +9319,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="77" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="77" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A77" t="s">
         <v>18</v>
       </c>
@@ -9347,7 +9372,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="78" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="78" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A78" t="s">
         <v>18</v>
       </c>
@@ -9400,7 +9425,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="79" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="79" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A79" t="s">
         <v>18</v>
       </c>
@@ -9453,7 +9478,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="80" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="80" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A80" t="s">
         <v>18</v>
       </c>
@@ -9506,7 +9531,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="81" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="81" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A81" t="s">
         <v>18</v>
       </c>
@@ -9559,7 +9584,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="82" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="82" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A82" t="s">
         <v>18</v>
       </c>
@@ -9612,7 +9637,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="83" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="83" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A83" t="s">
         <v>18</v>
       </c>
@@ -9665,7 +9690,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="84" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="84" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A84" t="s">
         <v>18</v>
       </c>
@@ -9718,7 +9743,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="85" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="85" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A85" t="s">
         <v>18</v>
       </c>
@@ -9771,7 +9796,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="86" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="86" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A86" t="s">
         <v>18</v>
       </c>
@@ -9824,7 +9849,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="87" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="87" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A87" t="s">
         <v>18</v>
       </c>
@@ -9877,7 +9902,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="88" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="88" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A88" t="s">
         <v>18</v>
       </c>
@@ -9930,7 +9955,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="89" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="89" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A89" t="s">
         <v>18</v>
       </c>
@@ -9983,7 +10008,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="90" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="90" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A90" t="s">
         <v>18</v>
       </c>
@@ -10036,7 +10061,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="91" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="91" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A91" t="s">
         <v>18</v>
       </c>
@@ -10089,7 +10114,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="92" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="92" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A92" t="s">
         <v>18</v>
       </c>
@@ -10142,7 +10167,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="93" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="93" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A93" t="s">
         <v>18</v>
       </c>
@@ -10195,7 +10220,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="94" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="94" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A94" t="s">
         <v>18</v>
       </c>
@@ -10248,7 +10273,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="95" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="95" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A95" t="s">
         <v>18</v>
       </c>
@@ -10301,7 +10326,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="96" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="96" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A96" t="s">
         <v>18</v>
       </c>
@@ -10354,7 +10379,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="97" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="97" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A97" t="s">
         <v>18</v>
       </c>
@@ -10407,7 +10432,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="98" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="98" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A98" t="s">
         <v>18</v>
       </c>
@@ -10460,7 +10485,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="99" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="99" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A99" t="s">
         <v>18</v>
       </c>
@@ -10513,7 +10538,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="100" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="100" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A100" t="s">
         <v>18</v>
       </c>
@@ -10566,7 +10591,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="101" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="101" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A101" t="s">
         <v>18</v>
       </c>
@@ -10619,7 +10644,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="102" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="102" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A102" t="s">
         <v>18</v>
       </c>
@@ -10672,7 +10697,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="103" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="103" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A103" t="s">
         <v>18</v>
       </c>
@@ -10725,7 +10750,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="104" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="104" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A104" t="s">
         <v>18</v>
       </c>
@@ -10778,7 +10803,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="105" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="105" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A105" t="s">
         <v>18</v>
       </c>
@@ -10831,7 +10856,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="106" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="106" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A106" t="s">
         <v>18</v>
       </c>
@@ -10884,7 +10909,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="107" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="107" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A107" t="s">
         <v>18</v>
       </c>
@@ -10937,7 +10962,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="108" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="108" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A108" t="s">
         <v>18</v>
       </c>
@@ -10990,7 +11015,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="109" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="109" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A109" t="s">
         <v>18</v>
       </c>
@@ -11043,7 +11068,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="110" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="110" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A110" t="s">
         <v>18</v>
       </c>
@@ -11096,7 +11121,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="111" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="111" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A111" t="s">
         <v>18</v>
       </c>
@@ -11149,7 +11174,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="112" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="112" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A112" t="s">
         <v>18</v>
       </c>
@@ -11202,7 +11227,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="113" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="113" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A113" t="s">
         <v>18</v>
       </c>
@@ -11255,7 +11280,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="114" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="114" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A114" t="s">
         <v>18</v>
       </c>
@@ -11308,7 +11333,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="115" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="115" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A115" t="s">
         <v>18</v>
       </c>
@@ -11361,7 +11386,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="116" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="116" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A116" t="s">
         <v>18</v>
       </c>
@@ -11414,7 +11439,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="117" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="117" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A117" t="s">
         <v>18</v>
       </c>
@@ -11467,7 +11492,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="118" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="118" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A118" t="s">
         <v>18</v>
       </c>
@@ -11520,7 +11545,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="119" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="119" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A119" t="s">
         <v>18</v>
       </c>
@@ -11573,7 +11598,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="120" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="120" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A120" t="s">
         <v>18</v>
       </c>
@@ -11626,7 +11651,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="121" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="121" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A121" t="s">
         <v>18</v>
       </c>
@@ -11679,7 +11704,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="122" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="122" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A122" t="s">
         <v>18</v>
       </c>
@@ -11732,7 +11757,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="123" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="123" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A123" t="s">
         <v>18</v>
       </c>
@@ -11785,7 +11810,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="124" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="124" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A124" t="s">
         <v>18</v>
       </c>
@@ -11838,7 +11863,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="125" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="125" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A125" t="s">
         <v>18</v>
       </c>
@@ -11891,7 +11916,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="126" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="126" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A126" t="s">
         <v>18</v>
       </c>
@@ -11944,7 +11969,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="127" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="127" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A127" t="s">
         <v>18</v>
       </c>
@@ -11997,7 +12022,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="128" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="128" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A128" t="s">
         <v>18</v>
       </c>
@@ -12050,7 +12075,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="129" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="129" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A129" t="s">
         <v>18</v>
       </c>
@@ -12103,7 +12128,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="130" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="130" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A130" t="s">
         <v>18</v>
       </c>
@@ -12156,7 +12181,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="131" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="131" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A131" t="s">
         <v>18</v>
       </c>
@@ -12209,7 +12234,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="132" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="132" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A132" t="s">
         <v>18</v>
       </c>
@@ -12262,7 +12287,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="133" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="133" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A133" t="s">
         <v>18</v>
       </c>
@@ -12315,7 +12340,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="134" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="134" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A134" t="s">
         <v>18</v>
       </c>
@@ -12368,7 +12393,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="135" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="135" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A135" t="s">
         <v>18</v>
       </c>
@@ -12421,7 +12446,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="136" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="136" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A136" t="s">
         <v>18</v>
       </c>
@@ -12474,7 +12499,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="137" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="137" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A137" t="s">
         <v>18</v>
       </c>
@@ -12527,7 +12552,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="138" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="138" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A138" t="s">
         <v>18</v>
       </c>
@@ -12580,7 +12605,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="139" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="139" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A139" t="s">
         <v>18</v>
       </c>
@@ -12633,7 +12658,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="140" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="140" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A140" t="s">
         <v>18</v>
       </c>
@@ -12686,7 +12711,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="141" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="141" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A141" t="s">
         <v>18</v>
       </c>
@@ -12739,7 +12764,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="142" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="142" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A142" t="s">
         <v>18</v>
       </c>
@@ -12792,7 +12817,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="143" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="143" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A143" t="s">
         <v>18</v>
       </c>
@@ -12845,7 +12870,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="144" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="144" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A144" t="s">
         <v>18</v>
       </c>
@@ -12898,7 +12923,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="145" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="145" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A145" t="s">
         <v>18</v>
       </c>
@@ -12951,7 +12976,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="146" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="146" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A146" t="s">
         <v>18</v>
       </c>
@@ -13004,7 +13029,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="147" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="147" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A147" t="s">
         <v>18</v>
       </c>
@@ -13057,7 +13082,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="148" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="148" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A148" t="s">
         <v>18</v>
       </c>
@@ -13110,7 +13135,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="149" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="149" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A149" t="s">
         <v>18</v>
       </c>
@@ -13163,7 +13188,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="150" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="150" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A150" t="s">
         <v>18</v>
       </c>
@@ -13216,7 +13241,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="151" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="151" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A151" t="s">
         <v>18</v>
       </c>
@@ -13269,7 +13294,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="152" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="152" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A152" t="s">
         <v>18</v>
       </c>
@@ -13322,7 +13347,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="153" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="153" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A153" t="s">
         <v>18</v>
       </c>
@@ -13375,7 +13400,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="154" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="154" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A154" t="s">
         <v>18</v>
       </c>
@@ -13428,7 +13453,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="155" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="155" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A155" t="s">
         <v>18</v>
       </c>
@@ -13481,7 +13506,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="156" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="156" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A156" t="s">
         <v>18</v>
       </c>
@@ -13534,7 +13559,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="157" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="157" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A157" t="s">
         <v>18</v>
       </c>
@@ -13587,7 +13612,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="158" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="158" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A158" t="s">
         <v>18</v>
       </c>
@@ -13640,7 +13665,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="159" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="159" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A159" t="s">
         <v>18</v>
       </c>
@@ -13693,7 +13718,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="160" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="160" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A160" t="s">
         <v>18</v>
       </c>
@@ -13746,7 +13771,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="161" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="161" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A161" t="s">
         <v>18</v>
       </c>
@@ -13799,7 +13824,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="162" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="162" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A162" t="s">
         <v>18</v>
       </c>
@@ -13852,7 +13877,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="163" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="163" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A163" t="s">
         <v>18</v>
       </c>
@@ -13905,7 +13930,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="164" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="164" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A164" t="s">
         <v>18</v>
       </c>
@@ -13958,7 +13983,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="165" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="165" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A165" t="s">
         <v>18</v>
       </c>
@@ -14011,7 +14036,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="166" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="166" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A166" t="s">
         <v>18</v>
       </c>
@@ -14064,7 +14089,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="167" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="167" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A167" t="s">
         <v>18</v>
       </c>
@@ -14117,7 +14142,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="168" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="168" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A168" t="s">
         <v>18</v>
       </c>
@@ -14170,7 +14195,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="169" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="169" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A169" t="s">
         <v>18</v>
       </c>
@@ -14223,7 +14248,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="170" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="170" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A170" t="s">
         <v>18</v>
       </c>
@@ -14276,7 +14301,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="171" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="171" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A171" t="s">
         <v>18</v>
       </c>
@@ -14329,7 +14354,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="172" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="172" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A172" t="s">
         <v>18</v>
       </c>
@@ -14382,7 +14407,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="173" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="173" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A173" t="s">
         <v>18</v>
       </c>
@@ -14435,700 +14460,700 @@
         <v>1</v>
       </c>
     </row>
-    <row r="174" spans="1:17" x14ac:dyDescent="0.3">
-      <c r="A174" s="6" t="s">
-        <v>18</v>
-      </c>
-      <c r="B174" s="6" t="s">
-        <v>19</v>
-      </c>
-      <c r="C174" s="6" t="s">
-        <v>20</v>
-      </c>
-      <c r="D174" s="6">
-        <v>-1</v>
-      </c>
-      <c r="E174" s="6" t="s">
+    <row r="174" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A174" s="7" t="s">
+        <v>18</v>
+      </c>
+      <c r="B174" s="7" t="s">
+        <v>19</v>
+      </c>
+      <c r="C174" s="7" t="s">
+        <v>20</v>
+      </c>
+      <c r="D174" s="7">
+        <v>-1</v>
+      </c>
+      <c r="E174" s="7" t="s">
         <v>61</v>
       </c>
-      <c r="F174" s="6">
-        <v>128</v>
-      </c>
-      <c r="G174" s="6" t="s">
-        <v>22</v>
-      </c>
-      <c r="H174" s="7">
+      <c r="F174" s="7">
+        <v>128</v>
+      </c>
+      <c r="G174" s="7" t="s">
+        <v>22</v>
+      </c>
+      <c r="H174" s="8">
         <v>45560</v>
       </c>
-      <c r="I174" s="6" t="s">
-        <v>23</v>
-      </c>
-      <c r="J174" s="6" t="s">
-        <v>24</v>
-      </c>
-      <c r="K174" s="6" t="s">
+      <c r="I174" s="7" t="s">
+        <v>23</v>
+      </c>
+      <c r="J174" s="7" t="s">
+        <v>24</v>
+      </c>
+      <c r="K174" s="7" t="s">
         <v>59</v>
       </c>
-      <c r="L174" s="6" t="s">
+      <c r="L174" s="7" t="s">
         <v>60</v>
       </c>
-      <c r="M174" s="6" t="s">
+      <c r="M174" s="7" t="s">
         <v>32</v>
       </c>
-      <c r="N174" s="6" t="s">
+      <c r="N174" s="7" t="s">
         <v>28</v>
       </c>
-      <c r="O174" s="6" t="s">
-        <v>29</v>
-      </c>
-      <c r="P174" s="6" t="s">
-        <v>29</v>
-      </c>
-      <c r="Q174" s="6">
+      <c r="O174" s="7" t="s">
+        <v>29</v>
+      </c>
+      <c r="P174" s="7" t="s">
+        <v>29</v>
+      </c>
+      <c r="Q174" s="7">
         <v>0</v>
       </c>
     </row>
-    <row r="175" spans="1:17" x14ac:dyDescent="0.3">
-      <c r="A175" s="6" t="s">
-        <v>18</v>
-      </c>
-      <c r="B175" s="6" t="s">
-        <v>19</v>
-      </c>
-      <c r="C175" s="6" t="s">
-        <v>20</v>
-      </c>
-      <c r="D175" s="6">
-        <v>-1</v>
-      </c>
-      <c r="E175" s="6" t="s">
+    <row r="175" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A175" s="7" t="s">
+        <v>18</v>
+      </c>
+      <c r="B175" s="7" t="s">
+        <v>19</v>
+      </c>
+      <c r="C175" s="7" t="s">
+        <v>20</v>
+      </c>
+      <c r="D175" s="7">
+        <v>-1</v>
+      </c>
+      <c r="E175" s="7" t="s">
         <v>64</v>
       </c>
-      <c r="F175" s="6">
+      <c r="F175" s="7">
+        <v>128</v>
+      </c>
+      <c r="G175" s="7" t="s">
+        <v>22</v>
+      </c>
+      <c r="H175" s="8">
+        <v>45560</v>
+      </c>
+      <c r="I175" s="7" t="s">
+        <v>23</v>
+      </c>
+      <c r="J175" s="7" t="s">
+        <v>24</v>
+      </c>
+      <c r="K175" s="7" t="s">
+        <v>49</v>
+      </c>
+      <c r="L175" s="7" t="s">
+        <v>50</v>
+      </c>
+      <c r="M175" s="7" t="s">
+        <v>27</v>
+      </c>
+      <c r="N175" s="7" t="s">
+        <v>28</v>
+      </c>
+      <c r="O175" s="7" t="s">
+        <v>29</v>
+      </c>
+      <c r="P175" s="7" t="s">
+        <v>29</v>
+      </c>
+      <c r="Q175" s="7">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="176" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A176" s="7" t="s">
+        <v>18</v>
+      </c>
+      <c r="B176" s="7" t="s">
+        <v>19</v>
+      </c>
+      <c r="C176" s="7" t="s">
+        <v>20</v>
+      </c>
+      <c r="D176" s="7">
+        <v>-1</v>
+      </c>
+      <c r="E176" s="7" t="s">
+        <v>21</v>
+      </c>
+      <c r="F176" s="7">
         <v>64</v>
       </c>
-      <c r="G175" s="6" t="s">
-        <v>22</v>
-      </c>
-      <c r="H175" s="7">
+      <c r="G176" s="7" t="s">
+        <v>22</v>
+      </c>
+      <c r="H176" s="8">
+        <v>45561</v>
+      </c>
+      <c r="I176" s="7" t="s">
+        <v>23</v>
+      </c>
+      <c r="J176" s="7" t="s">
+        <v>24</v>
+      </c>
+      <c r="K176" s="7" t="s">
+        <v>67</v>
+      </c>
+      <c r="L176" s="7" t="s">
+        <v>68</v>
+      </c>
+      <c r="M176" s="7" t="s">
+        <v>35</v>
+      </c>
+      <c r="N176" s="7" t="s">
+        <v>36</v>
+      </c>
+      <c r="O176" s="7" t="s">
+        <v>29</v>
+      </c>
+      <c r="P176" s="7" t="s">
+        <v>41</v>
+      </c>
+      <c r="Q176" s="7">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="177" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A177" s="7" t="s">
+        <v>18</v>
+      </c>
+      <c r="B177" s="7" t="s">
+        <v>19</v>
+      </c>
+      <c r="C177" s="7" t="s">
+        <v>20</v>
+      </c>
+      <c r="D177" s="7">
+        <v>-1</v>
+      </c>
+      <c r="E177" s="7" t="s">
+        <v>61</v>
+      </c>
+      <c r="F177" s="7">
+        <v>64</v>
+      </c>
+      <c r="G177" s="7" t="s">
+        <v>22</v>
+      </c>
+      <c r="H177" s="8">
+        <v>45561</v>
+      </c>
+      <c r="I177" s="7" t="s">
+        <v>23</v>
+      </c>
+      <c r="J177" s="7" t="s">
+        <v>24</v>
+      </c>
+      <c r="K177" s="7" t="s">
+        <v>67</v>
+      </c>
+      <c r="L177" s="7" t="s">
+        <v>68</v>
+      </c>
+      <c r="M177" s="7" t="s">
+        <v>35</v>
+      </c>
+      <c r="N177" s="7" t="s">
+        <v>36</v>
+      </c>
+      <c r="O177" s="7" t="s">
+        <v>29</v>
+      </c>
+      <c r="P177" s="7" t="s">
+        <v>41</v>
+      </c>
+      <c r="Q177" s="7">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="178" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A178" s="7" t="s">
+        <v>18</v>
+      </c>
+      <c r="B178" s="7" t="s">
+        <v>19</v>
+      </c>
+      <c r="C178" s="7" t="s">
+        <v>20</v>
+      </c>
+      <c r="D178" s="7">
+        <v>-1</v>
+      </c>
+      <c r="E178" s="7" t="s">
+        <v>61</v>
+      </c>
+      <c r="F178" s="7">
+        <v>128</v>
+      </c>
+      <c r="G178" s="7" t="s">
+        <v>22</v>
+      </c>
+      <c r="H178" s="8">
         <v>45560</v>
       </c>
-      <c r="I175" s="6" t="s">
-        <v>23</v>
-      </c>
-      <c r="J175" s="6" t="s">
-        <v>24</v>
-      </c>
-      <c r="K175" s="6" t="s">
-        <v>49</v>
-      </c>
-      <c r="L175" s="6" t="s">
-        <v>50</v>
-      </c>
-      <c r="M175" s="6" t="s">
-        <v>27</v>
-      </c>
-      <c r="N175" s="6" t="s">
-        <v>28</v>
-      </c>
-      <c r="O175" s="6" t="s">
-        <v>29</v>
-      </c>
-      <c r="P175" s="6" t="s">
-        <v>29</v>
-      </c>
-      <c r="Q175" s="6">
+      <c r="I178" s="7" t="s">
+        <v>23</v>
+      </c>
+      <c r="J178" s="7" t="s">
+        <v>24</v>
+      </c>
+      <c r="K178" s="7" t="s">
+        <v>46</v>
+      </c>
+      <c r="L178" s="7" t="s">
+        <v>47</v>
+      </c>
+      <c r="M178" s="7" t="s">
+        <v>35</v>
+      </c>
+      <c r="N178" s="7" t="s">
+        <v>36</v>
+      </c>
+      <c r="O178" s="7" t="s">
+        <v>29</v>
+      </c>
+      <c r="P178" s="7" t="s">
+        <v>41</v>
+      </c>
+      <c r="Q178" s="7">
         <v>0</v>
       </c>
     </row>
-    <row r="176" spans="1:17" x14ac:dyDescent="0.3">
-      <c r="A176" s="6" t="s">
-        <v>18</v>
-      </c>
-      <c r="B176" s="6" t="s">
-        <v>19</v>
-      </c>
-      <c r="C176" s="6" t="s">
-        <v>20</v>
-      </c>
-      <c r="D176" s="6">
-        <v>-1</v>
-      </c>
-      <c r="E176" s="6" t="s">
+    <row r="179" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A179" s="7" t="s">
+        <v>18</v>
+      </c>
+      <c r="B179" s="7" t="s">
+        <v>19</v>
+      </c>
+      <c r="C179" s="7" t="s">
+        <v>20</v>
+      </c>
+      <c r="D179" s="7">
+        <v>-1</v>
+      </c>
+      <c r="E179" s="7" t="s">
+        <v>64</v>
+      </c>
+      <c r="F179" s="7">
+        <v>128</v>
+      </c>
+      <c r="G179" s="7" t="s">
+        <v>22</v>
+      </c>
+      <c r="H179" s="8">
+        <v>45560</v>
+      </c>
+      <c r="I179" s="7" t="s">
+        <v>23</v>
+      </c>
+      <c r="J179" s="7" t="s">
+        <v>24</v>
+      </c>
+      <c r="K179" s="7" t="s">
+        <v>46</v>
+      </c>
+      <c r="L179" s="7" t="s">
+        <v>47</v>
+      </c>
+      <c r="M179" s="7" t="s">
+        <v>35</v>
+      </c>
+      <c r="N179" s="7" t="s">
+        <v>36</v>
+      </c>
+      <c r="O179" s="7" t="s">
+        <v>29</v>
+      </c>
+      <c r="P179" s="7" t="s">
+        <v>41</v>
+      </c>
+      <c r="Q179" s="7">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="180" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A180" s="7" t="s">
+        <v>18</v>
+      </c>
+      <c r="B180" s="7" t="s">
+        <v>19</v>
+      </c>
+      <c r="C180" s="7" t="s">
+        <v>20</v>
+      </c>
+      <c r="D180" s="7">
+        <v>-1</v>
+      </c>
+      <c r="E180" s="7" t="s">
         <v>21</v>
       </c>
-      <c r="F176" s="6">
-        <v>128</v>
-      </c>
-      <c r="G176" s="6" t="s">
-        <v>22</v>
-      </c>
-      <c r="H176" s="7">
+      <c r="F180" s="7">
+        <v>128</v>
+      </c>
+      <c r="G180" s="7" t="s">
+        <v>22</v>
+      </c>
+      <c r="H180" s="8">
         <v>45561</v>
       </c>
-      <c r="I176" s="6" t="s">
-        <v>23</v>
-      </c>
-      <c r="J176" s="6" t="s">
-        <v>24</v>
-      </c>
-      <c r="K176" s="6" t="s">
-        <v>67</v>
-      </c>
-      <c r="L176" s="6" t="s">
-        <v>68</v>
-      </c>
-      <c r="M176" s="6" t="s">
-        <v>35</v>
-      </c>
-      <c r="N176" s="6" t="s">
+      <c r="I180" s="7" t="s">
+        <v>23</v>
+      </c>
+      <c r="J180" s="7" t="s">
+        <v>24</v>
+      </c>
+      <c r="K180" s="7" t="s">
+        <v>62</v>
+      </c>
+      <c r="L180" s="7" t="s">
+        <v>63</v>
+      </c>
+      <c r="M180" s="7" t="s">
+        <v>44</v>
+      </c>
+      <c r="N180" s="7" t="s">
+        <v>45</v>
+      </c>
+      <c r="O180" s="7" t="s">
+        <v>29</v>
+      </c>
+      <c r="P180" s="7" t="s">
+        <v>29</v>
+      </c>
+      <c r="Q180" s="7">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="181" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A181" s="7" t="s">
+        <v>18</v>
+      </c>
+      <c r="B181" s="7" t="s">
+        <v>19</v>
+      </c>
+      <c r="C181" s="7" t="s">
+        <v>20</v>
+      </c>
+      <c r="D181" s="7">
+        <v>-1</v>
+      </c>
+      <c r="E181" s="7" t="s">
+        <v>64</v>
+      </c>
+      <c r="F181" s="7">
+        <v>128</v>
+      </c>
+      <c r="G181" s="7" t="s">
+        <v>22</v>
+      </c>
+      <c r="H181" s="8">
+        <v>45561</v>
+      </c>
+      <c r="I181" s="7" t="s">
+        <v>23</v>
+      </c>
+      <c r="J181" s="7" t="s">
+        <v>24</v>
+      </c>
+      <c r="K181" s="7" t="s">
+        <v>62</v>
+      </c>
+      <c r="L181" s="7" t="s">
+        <v>63</v>
+      </c>
+      <c r="M181" s="7" t="s">
+        <v>44</v>
+      </c>
+      <c r="N181" s="7" t="s">
+        <v>45</v>
+      </c>
+      <c r="O181" s="7" t="s">
+        <v>29</v>
+      </c>
+      <c r="P181" s="7" t="s">
+        <v>29</v>
+      </c>
+      <c r="Q181" s="7">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="182" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A182" s="7" t="s">
+        <v>18</v>
+      </c>
+      <c r="B182" s="7" t="s">
+        <v>19</v>
+      </c>
+      <c r="C182" s="7" t="s">
+        <v>20</v>
+      </c>
+      <c r="D182" s="7">
+        <v>-1</v>
+      </c>
+      <c r="E182" s="7" t="s">
+        <v>21</v>
+      </c>
+      <c r="F182" s="7">
+        <v>64</v>
+      </c>
+      <c r="G182" s="7" t="s">
+        <v>22</v>
+      </c>
+      <c r="H182" s="8">
+        <v>45561</v>
+      </c>
+      <c r="I182" s="7" t="s">
+        <v>23</v>
+      </c>
+      <c r="J182" s="7" t="s">
+        <v>24</v>
+      </c>
+      <c r="K182" s="7" t="s">
+        <v>65</v>
+      </c>
+      <c r="L182" s="7" t="s">
+        <v>66</v>
+      </c>
+      <c r="M182" s="7" t="s">
+        <v>58</v>
+      </c>
+      <c r="N182" s="7" t="s">
         <v>36</v>
       </c>
-      <c r="O176" s="6" t="s">
-        <v>29</v>
-      </c>
-      <c r="P176" s="6" t="s">
-        <v>41</v>
-      </c>
-      <c r="Q176" s="6">
+      <c r="O182" s="7" t="s">
+        <v>29</v>
+      </c>
+      <c r="P182" s="7" t="s">
+        <v>37</v>
+      </c>
+      <c r="Q182" s="7">
         <v>0</v>
       </c>
     </row>
-    <row r="177" spans="1:17" x14ac:dyDescent="0.3">
-      <c r="A177" s="6" t="s">
-        <v>18</v>
-      </c>
-      <c r="B177" s="6" t="s">
-        <v>19</v>
-      </c>
-      <c r="C177" s="6" t="s">
-        <v>20</v>
-      </c>
-      <c r="D177" s="6">
-        <v>-1</v>
-      </c>
-      <c r="E177" s="6" t="s">
+    <row r="183" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A183" s="7" t="s">
+        <v>18</v>
+      </c>
+      <c r="B183" s="7" t="s">
+        <v>19</v>
+      </c>
+      <c r="C183" s="7" t="s">
+        <v>20</v>
+      </c>
+      <c r="D183" s="7">
+        <v>-1</v>
+      </c>
+      <c r="E183" s="7" t="s">
         <v>61</v>
       </c>
-      <c r="F177" s="6">
-        <v>128</v>
-      </c>
-      <c r="G177" s="6" t="s">
-        <v>22</v>
-      </c>
-      <c r="H177" s="7">
+      <c r="F183" s="7">
+        <v>64</v>
+      </c>
+      <c r="G183" s="7" t="s">
+        <v>22</v>
+      </c>
+      <c r="H183" s="8">
         <v>45561</v>
       </c>
-      <c r="I177" s="6" t="s">
-        <v>23</v>
-      </c>
-      <c r="J177" s="6" t="s">
-        <v>24</v>
-      </c>
-      <c r="K177" s="6" t="s">
-        <v>67</v>
-      </c>
-      <c r="L177" s="6" t="s">
-        <v>68</v>
-      </c>
-      <c r="M177" s="6" t="s">
-        <v>35</v>
-      </c>
-      <c r="N177" s="6" t="s">
+      <c r="I183" s="7" t="s">
+        <v>23</v>
+      </c>
+      <c r="J183" s="7" t="s">
+        <v>24</v>
+      </c>
+      <c r="K183" s="7" t="s">
+        <v>65</v>
+      </c>
+      <c r="L183" s="7" t="s">
+        <v>66</v>
+      </c>
+      <c r="M183" s="7" t="s">
+        <v>58</v>
+      </c>
+      <c r="N183" s="7" t="s">
         <v>36</v>
       </c>
-      <c r="O177" s="6" t="s">
-        <v>29</v>
-      </c>
-      <c r="P177" s="6" t="s">
-        <v>41</v>
-      </c>
-      <c r="Q177" s="6">
+      <c r="O183" s="7" t="s">
+        <v>29</v>
+      </c>
+      <c r="P183" s="7" t="s">
+        <v>37</v>
+      </c>
+      <c r="Q183" s="7">
         <v>0</v>
       </c>
     </row>
-    <row r="178" spans="1:17" x14ac:dyDescent="0.3">
-      <c r="A178" s="6" t="s">
-        <v>18</v>
-      </c>
-      <c r="B178" s="6" t="s">
-        <v>19</v>
-      </c>
-      <c r="C178" s="6" t="s">
-        <v>20</v>
-      </c>
-      <c r="D178" s="6">
-        <v>-1</v>
-      </c>
-      <c r="E178" s="6" t="s">
+    <row r="184" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A184" s="7" t="s">
+        <v>18</v>
+      </c>
+      <c r="B184" s="7" t="s">
+        <v>19</v>
+      </c>
+      <c r="C184" s="7" t="s">
+        <v>20</v>
+      </c>
+      <c r="D184" s="7">
+        <v>-1</v>
+      </c>
+      <c r="E184" s="7" t="s">
         <v>61</v>
       </c>
-      <c r="F178" s="6">
-        <v>128</v>
-      </c>
-      <c r="G178" s="6" t="s">
-        <v>22</v>
-      </c>
-      <c r="H178" s="7">
-        <v>45560</v>
-      </c>
-      <c r="I178" s="6" t="s">
-        <v>23</v>
-      </c>
-      <c r="J178" s="6" t="s">
-        <v>24</v>
-      </c>
-      <c r="K178" s="6" t="s">
-        <v>46</v>
-      </c>
-      <c r="L178" s="6" t="s">
-        <v>47</v>
-      </c>
-      <c r="M178" s="6" t="s">
-        <v>35</v>
-      </c>
-      <c r="N178" s="6" t="s">
+      <c r="F184" s="7">
+        <v>128</v>
+      </c>
+      <c r="G184" s="7" t="s">
+        <v>22</v>
+      </c>
+      <c r="H184" s="8">
+        <v>45561</v>
+      </c>
+      <c r="I184" s="7" t="s">
+        <v>23</v>
+      </c>
+      <c r="J184" s="7" t="s">
+        <v>24</v>
+      </c>
+      <c r="K184" s="7" t="s">
+        <v>56</v>
+      </c>
+      <c r="L184" s="7" t="s">
+        <v>57</v>
+      </c>
+      <c r="M184" s="7" t="s">
+        <v>58</v>
+      </c>
+      <c r="N184" s="7" t="s">
         <v>36</v>
       </c>
-      <c r="O178" s="6" t="s">
-        <v>29</v>
-      </c>
-      <c r="P178" s="6" t="s">
-        <v>41</v>
-      </c>
-      <c r="Q178" s="6">
+      <c r="O184" s="7" t="s">
+        <v>29</v>
+      </c>
+      <c r="P184" s="7" t="s">
+        <v>37</v>
+      </c>
+      <c r="Q184" s="7">
         <v>0</v>
       </c>
     </row>
-    <row r="179" spans="1:17" x14ac:dyDescent="0.3">
-      <c r="A179" s="6" t="s">
-        <v>18</v>
-      </c>
-      <c r="B179" s="6" t="s">
-        <v>19</v>
-      </c>
-      <c r="C179" s="6" t="s">
-        <v>20</v>
-      </c>
-      <c r="D179" s="6">
-        <v>-1</v>
-      </c>
-      <c r="E179" s="6" t="s">
+    <row r="185" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A185" s="7" t="s">
+        <v>18</v>
+      </c>
+      <c r="B185" s="7" t="s">
+        <v>19</v>
+      </c>
+      <c r="C185" s="7" t="s">
+        <v>20</v>
+      </c>
+      <c r="D185" s="7">
+        <v>-1</v>
+      </c>
+      <c r="E185" s="7" t="s">
         <v>64</v>
       </c>
-      <c r="F179" s="6">
-        <v>64</v>
-      </c>
-      <c r="G179" s="6" t="s">
-        <v>22</v>
-      </c>
-      <c r="H179" s="7">
-        <v>45560</v>
-      </c>
-      <c r="I179" s="6" t="s">
-        <v>23</v>
-      </c>
-      <c r="J179" s="6" t="s">
-        <v>24</v>
-      </c>
-      <c r="K179" s="6" t="s">
-        <v>46</v>
-      </c>
-      <c r="L179" s="6" t="s">
-        <v>47</v>
-      </c>
-      <c r="M179" s="6" t="s">
-        <v>35</v>
-      </c>
-      <c r="N179" s="6" t="s">
+      <c r="F185" s="7">
+        <v>128</v>
+      </c>
+      <c r="G185" s="7" t="s">
+        <v>22</v>
+      </c>
+      <c r="H185" s="8">
+        <v>45561</v>
+      </c>
+      <c r="I185" s="7" t="s">
+        <v>23</v>
+      </c>
+      <c r="J185" s="7" t="s">
+        <v>24</v>
+      </c>
+      <c r="K185" s="7" t="s">
+        <v>56</v>
+      </c>
+      <c r="L185" s="7" t="s">
+        <v>57</v>
+      </c>
+      <c r="M185" s="7" t="s">
+        <v>58</v>
+      </c>
+      <c r="N185" s="7" t="s">
         <v>36</v>
       </c>
-      <c r="O179" s="6" t="s">
-        <v>29</v>
-      </c>
-      <c r="P179" s="6" t="s">
-        <v>41</v>
-      </c>
-      <c r="Q179" s="6">
+      <c r="O185" s="7" t="s">
+        <v>29</v>
+      </c>
+      <c r="P185" s="7" t="s">
+        <v>37</v>
+      </c>
+      <c r="Q185" s="7">
         <v>0</v>
       </c>
     </row>
-    <row r="180" spans="1:17" x14ac:dyDescent="0.3">
-      <c r="A180" s="6" t="s">
-        <v>18</v>
-      </c>
-      <c r="B180" s="6" t="s">
-        <v>19</v>
-      </c>
-      <c r="C180" s="6" t="s">
-        <v>20</v>
-      </c>
-      <c r="D180" s="6">
-        <v>-1</v>
-      </c>
-      <c r="E180" s="6" t="s">
-        <v>21</v>
-      </c>
-      <c r="F180" s="6">
-        <v>128</v>
-      </c>
-      <c r="G180" s="6" t="s">
-        <v>22</v>
-      </c>
-      <c r="H180" s="7">
-        <v>45561</v>
-      </c>
-      <c r="I180" s="6" t="s">
-        <v>23</v>
-      </c>
-      <c r="J180" s="6" t="s">
-        <v>24</v>
-      </c>
-      <c r="K180" s="6" t="s">
-        <v>62</v>
-      </c>
-      <c r="L180" s="6" t="s">
-        <v>63</v>
-      </c>
-      <c r="M180" s="6" t="s">
-        <v>44</v>
-      </c>
-      <c r="N180" s="6" t="s">
-        <v>45</v>
-      </c>
-      <c r="O180" s="6" t="s">
-        <v>29</v>
-      </c>
-      <c r="P180" s="6" t="s">
-        <v>29</v>
-      </c>
-      <c r="Q180" s="6">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="181" spans="1:17" x14ac:dyDescent="0.3">
-      <c r="A181" s="6" t="s">
-        <v>18</v>
-      </c>
-      <c r="B181" s="6" t="s">
-        <v>19</v>
-      </c>
-      <c r="C181" s="6" t="s">
-        <v>20</v>
-      </c>
-      <c r="D181" s="6">
-        <v>-1</v>
-      </c>
-      <c r="E181" s="6" t="s">
-        <v>64</v>
-      </c>
-      <c r="F181" s="6">
-        <v>64</v>
-      </c>
-      <c r="G181" s="6" t="s">
-        <v>22</v>
-      </c>
-      <c r="H181" s="7">
-        <v>45561</v>
-      </c>
-      <c r="I181" s="6" t="s">
-        <v>23</v>
-      </c>
-      <c r="J181" s="6" t="s">
-        <v>24</v>
-      </c>
-      <c r="K181" s="6" t="s">
-        <v>62</v>
-      </c>
-      <c r="L181" s="6" t="s">
-        <v>63</v>
-      </c>
-      <c r="M181" s="6" t="s">
-        <v>44</v>
-      </c>
-      <c r="N181" s="6" t="s">
-        <v>45</v>
-      </c>
-      <c r="O181" s="6" t="s">
-        <v>29</v>
-      </c>
-      <c r="P181" s="6" t="s">
-        <v>29</v>
-      </c>
-      <c r="Q181" s="6">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="182" spans="1:17" x14ac:dyDescent="0.3">
-      <c r="A182" s="6" t="s">
-        <v>18</v>
-      </c>
-      <c r="B182" s="6" t="s">
-        <v>19</v>
-      </c>
-      <c r="C182" s="6" t="s">
-        <v>20</v>
-      </c>
-      <c r="D182" s="6">
-        <v>-1</v>
-      </c>
-      <c r="E182" s="6" t="s">
-        <v>21</v>
-      </c>
-      <c r="F182" s="6">
-        <v>128</v>
-      </c>
-      <c r="G182" s="6" t="s">
-        <v>22</v>
-      </c>
-      <c r="H182" s="7">
-        <v>45561</v>
-      </c>
-      <c r="I182" s="6" t="s">
-        <v>23</v>
-      </c>
-      <c r="J182" s="6" t="s">
-        <v>24</v>
-      </c>
-      <c r="K182" s="6" t="s">
-        <v>65</v>
-      </c>
-      <c r="L182" s="6" t="s">
-        <v>66</v>
-      </c>
-      <c r="M182" s="6" t="s">
-        <v>58</v>
-      </c>
-      <c r="N182" s="6" t="s">
-        <v>36</v>
-      </c>
-      <c r="O182" s="6" t="s">
-        <v>29</v>
-      </c>
-      <c r="P182" s="6" t="s">
-        <v>37</v>
-      </c>
-      <c r="Q182" s="6">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="183" spans="1:17" x14ac:dyDescent="0.3">
-      <c r="A183" s="6" t="s">
-        <v>18</v>
-      </c>
-      <c r="B183" s="6" t="s">
-        <v>19</v>
-      </c>
-      <c r="C183" s="6" t="s">
-        <v>20</v>
-      </c>
-      <c r="D183" s="6">
-        <v>-1</v>
-      </c>
-      <c r="E183" s="6" t="s">
-        <v>61</v>
-      </c>
-      <c r="F183" s="6">
-        <v>128</v>
-      </c>
-      <c r="G183" s="6" t="s">
-        <v>22</v>
-      </c>
-      <c r="H183" s="7">
-        <v>45561</v>
-      </c>
-      <c r="I183" s="6" t="s">
-        <v>23</v>
-      </c>
-      <c r="J183" s="6" t="s">
-        <v>24</v>
-      </c>
-      <c r="K183" s="6" t="s">
-        <v>65</v>
-      </c>
-      <c r="L183" s="6" t="s">
-        <v>66</v>
-      </c>
-      <c r="M183" s="6" t="s">
-        <v>58</v>
-      </c>
-      <c r="N183" s="6" t="s">
-        <v>36</v>
-      </c>
-      <c r="O183" s="6" t="s">
-        <v>29</v>
-      </c>
-      <c r="P183" s="6" t="s">
-        <v>37</v>
-      </c>
-      <c r="Q183" s="6">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="184" spans="1:17" x14ac:dyDescent="0.3">
-      <c r="A184" s="6" t="s">
-        <v>18</v>
-      </c>
-      <c r="B184" s="6" t="s">
-        <v>19</v>
-      </c>
-      <c r="C184" s="6" t="s">
-        <v>20</v>
-      </c>
-      <c r="D184" s="6">
-        <v>-1</v>
-      </c>
-      <c r="E184" s="6" t="s">
-        <v>61</v>
-      </c>
-      <c r="F184" s="6">
-        <v>128</v>
-      </c>
-      <c r="G184" s="6" t="s">
-        <v>22</v>
-      </c>
-      <c r="H184" s="7">
-        <v>45561</v>
-      </c>
-      <c r="I184" s="6" t="s">
-        <v>23</v>
-      </c>
-      <c r="J184" s="6" t="s">
-        <v>24</v>
-      </c>
-      <c r="K184" s="6" t="s">
-        <v>56</v>
-      </c>
-      <c r="L184" s="6" t="s">
-        <v>57</v>
-      </c>
-      <c r="M184" s="6" t="s">
-        <v>58</v>
-      </c>
-      <c r="N184" s="6" t="s">
-        <v>36</v>
-      </c>
-      <c r="O184" s="6" t="s">
-        <v>29</v>
-      </c>
-      <c r="P184" s="6" t="s">
-        <v>37</v>
-      </c>
-      <c r="Q184" s="6">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="185" spans="1:17" x14ac:dyDescent="0.3">
-      <c r="A185" s="6" t="s">
-        <v>18</v>
-      </c>
-      <c r="B185" s="6" t="s">
-        <v>19</v>
-      </c>
-      <c r="C185" s="6" t="s">
-        <v>20</v>
-      </c>
-      <c r="D185" s="6">
-        <v>-1</v>
-      </c>
-      <c r="E185" s="6" t="s">
-        <v>64</v>
-      </c>
-      <c r="F185" s="6">
-        <v>64</v>
-      </c>
-      <c r="G185" s="6" t="s">
-        <v>22</v>
-      </c>
-      <c r="H185" s="7">
-        <v>45561</v>
-      </c>
-      <c r="I185" s="6" t="s">
-        <v>23</v>
-      </c>
-      <c r="J185" s="6" t="s">
-        <v>24</v>
-      </c>
-      <c r="K185" s="6" t="s">
-        <v>56</v>
-      </c>
-      <c r="L185" s="6" t="s">
-        <v>57</v>
-      </c>
-      <c r="M185" s="6" t="s">
-        <v>58</v>
-      </c>
-      <c r="N185" s="6" t="s">
-        <v>36</v>
-      </c>
-      <c r="O185" s="6" t="s">
-        <v>29</v>
-      </c>
-      <c r="P185" s="6" t="s">
-        <v>37</v>
-      </c>
-      <c r="Q185" s="6">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="186" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="186" spans="1:17" x14ac:dyDescent="0.25">
       <c r="H186" s="1"/>
     </row>
-    <row r="187" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="187" spans="1:17" x14ac:dyDescent="0.25">
       <c r="H187" s="1"/>
     </row>
-    <row r="188" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="188" spans="1:17" x14ac:dyDescent="0.25">
       <c r="H188" s="1"/>
     </row>
-    <row r="189" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="189" spans="1:17" x14ac:dyDescent="0.25">
       <c r="H189" s="1"/>
     </row>
-    <row r="190" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="190" spans="1:17" x14ac:dyDescent="0.25">
       <c r="H190" s="1"/>
     </row>
-    <row r="191" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="191" spans="1:17" x14ac:dyDescent="0.25">
       <c r="H191" s="1"/>
     </row>
-    <row r="192" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="192" spans="1:17" x14ac:dyDescent="0.25">
       <c r="H192" s="1"/>
     </row>
-    <row r="193" spans="8:8" x14ac:dyDescent="0.3">
+    <row r="193" spans="8:8" x14ac:dyDescent="0.25">
       <c r="H193" s="1"/>
     </row>
-    <row r="194" spans="8:8" x14ac:dyDescent="0.3">
+    <row r="194" spans="8:8" x14ac:dyDescent="0.25">
       <c r="H194" s="1"/>
     </row>
-    <row r="195" spans="8:8" x14ac:dyDescent="0.3">
+    <row r="195" spans="8:8" x14ac:dyDescent="0.25">
       <c r="H195" s="1"/>
     </row>
-    <row r="196" spans="8:8" x14ac:dyDescent="0.3">
+    <row r="196" spans="8:8" x14ac:dyDescent="0.25">
       <c r="H196" s="1"/>
     </row>
-    <row r="197" spans="8:8" x14ac:dyDescent="0.3">
+    <row r="197" spans="8:8" x14ac:dyDescent="0.25">
       <c r="H197" s="1"/>
     </row>
-    <row r="198" spans="8:8" x14ac:dyDescent="0.3">
+    <row r="198" spans="8:8" x14ac:dyDescent="0.25">
       <c r="H198" s="1"/>
     </row>
-    <row r="199" spans="8:8" x14ac:dyDescent="0.3">
+    <row r="199" spans="8:8" x14ac:dyDescent="0.25">
       <c r="H199" s="1"/>
     </row>
-    <row r="200" spans="8:8" x14ac:dyDescent="0.3">
+    <row r="200" spans="8:8" x14ac:dyDescent="0.25">
       <c r="H200" s="1"/>
     </row>
-    <row r="201" spans="8:8" x14ac:dyDescent="0.3">
+    <row r="201" spans="8:8" x14ac:dyDescent="0.25">
       <c r="H201" s="1"/>
     </row>
-    <row r="202" spans="8:8" x14ac:dyDescent="0.3">
+    <row r="202" spans="8:8" x14ac:dyDescent="0.25">
       <c r="H202" s="1"/>
     </row>
-    <row r="203" spans="8:8" x14ac:dyDescent="0.3">
+    <row r="203" spans="8:8" x14ac:dyDescent="0.25">
       <c r="H203" s="1"/>
     </row>
-    <row r="204" spans="8:8" x14ac:dyDescent="0.3">
+    <row r="204" spans="8:8" x14ac:dyDescent="0.25">
       <c r="H204" s="1"/>
     </row>
-    <row r="205" spans="8:8" x14ac:dyDescent="0.3">
+    <row r="205" spans="8:8" x14ac:dyDescent="0.25">
       <c r="H205" s="1"/>
     </row>
   </sheetData>

</xml_diff>